<commit_message>
feat: resto dos arquivos
</commit_message>
<xml_diff>
--- a/simulacaoes_/custo_robustez_C13/_lote_casos.xlsx
+++ b/simulacaoes_/custo_robustez_C13/_lote_casos.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,212 +417,212 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Comprimento das longarinas (cm)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Largura da pista disponível para longarinas (cm)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>['Circular']</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Tipo de seção do tabuleiro</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Carga permanente atuante no tabuleiro (kN/m²) excluso peso próprio (kPa)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Carga por roda (kN) (kN)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Carga de multidão (kN/m²) (kPa)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Distância entre eixos (m) do veículo tipo (m)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Classe de carregamento</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Classe de madeira</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Classe de umidade</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>γg - Carga permanente</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>γq - Carga variável</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>γwc - Cisalhamento</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>γwf - Flexão</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>ψ2</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Coeficiente para fluência Tabela 20 NBR 7190</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Percentual de robustez</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Densidade da madeira (kg/m³) da longarina (kg/m³)</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Resistência característica à flexão (MPa) da longarina (MPa)</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Resistência característica ao cisalhamento (MPa) da longarina (MPa)</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Módulo de elasticidade à flexão (GPa) da longarina (GPa)</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Densidade da madeira (kg/m³) do tabuleiro (kg/m³)</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Resistência característica à flexão (MPa) do tabuleiro (MPa)</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>cfg_d_min</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>cfg_d_max</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>cfg_bw_min</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>cfg_bw_max</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>cfg_h_min</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>cfg_h_max</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>cfg_esp_long_min</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>cfg_esp_long_max</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>cfg_esp_tab_min</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>cfg_esp_tab_max</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>cfg_pop_size</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>cfg_n_gen</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>cfg_n_checagens</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>cfg_sobol</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>cfg_sobol_n_samples</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>cfg_ativo</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>cfg_subdiretorio</t>
         </is>

</xml_diff>